<commit_message>
Nap DS 8 NV that + theme nau + file van phong
</commit_message>
<xml_diff>
--- a/File_VanPhong_NhapLich_XemCong.xlsx
+++ b/File_VanPhong_NhapLich_XemCong.xlsx
@@ -8,11 +8,13 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HUONGDAN" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LICHLAM" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BAOCAO_THANG" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DANHSACH" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LICHLAM" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BAOCAO_THANG" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'LICHLAM'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'DANHSACH'!$A$1:$C$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'LICHLAM'!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -464,7 +466,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ví dụ: NV001 | Tuấn Ngọc | T3 | Sáng | 08:00 | 10:30</t>
+          <t>Ví dụ: NV0101 | Mr. Ngọc | T3 | Sáng | 08:00 | 10:30</t>
         </is>
       </c>
     </row>
@@ -488,7 +490,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>XEM KẾT QUẢ: mở link web báo cáo (?page=baocao), gõ ngày kiểu 10/09/2026 để xem ngày, gõ NV001 09/2026 để xem tổng giờ tháng + trễ + quên RA + KPI.</t>
+          <t>XEM KẾT QUẢ: mở link web báo cáo (?page=baocao), gõ ngày kiểu 10/09/2026 để xem ngày, gõ mã NV + tháng kiểu NV0101 09/2026 để xem tổng giờ tháng + trễ + quên RA + KPI.</t>
         </is>
       </c>
     </row>
@@ -503,7 +505,185 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Mã NV</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Họ và tên</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Vai trò (Giáo viên / Văn phòng)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>NV0101</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Mr. Ngọc</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Giáo viên</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>NV0204</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Ms. Vân Anh</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Văn phòng</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>NV2707</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Mr. Đức Anh</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Giáo viên</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>NV1308</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Ms. Hồng Anh</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Giáo viên</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>NV0904</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Ms. Vân</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Giáo viên</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>NV2412</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ms. Trâm</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Giáo viên</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>NV2301</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Ms. Uyên Vi</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Giáo viên</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>NV0801</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Mr. Khôi</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Văn phòng</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C1"/>
+  <dataValidations count="1">
+    <dataValidation sqref="C2:C100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Giáo viên,Văn phòng"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -522,7 +702,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Họ và tên</t>
+          <t>Họ và tên (tự gõ lại cho dễ đọc)</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -549,12 +729,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>NV001</t>
+          <t>NV0101</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Tuấn Ngọc</t>
+          <t>Mr. Ngọc</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -581,12 +761,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>NV001</t>
+          <t>NV0101</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Tuấn Ngọc</t>
+          <t>Mr. Ngọc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -613,12 +793,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NV001</t>
+          <t>NV0101</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Tuấn Ngọc</t>
+          <t>Mr. Ngọc</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -641,6 +821,46 @@
           <t>11:30</t>
         </is>
       </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>
@@ -656,13 +876,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -720,12 +940,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>NV001</t>
+          <t>NV0101</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Tuấn Ngọc</t>
+          <t>Mr. Ngọc</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -740,9 +960,21 @@
       <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>NV0204</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Ms. Vân Anh</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>09/2026</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
@@ -752,17 +984,152 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ghi chú: số liệu trang này copy từ trang báo cáo web (?page=baocao), hoặc xem trực tiếp trên web.</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
+          <t>NV2707</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Mr. Đức Anh</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>09/2026</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>NV1308</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Ms. Hồng Anh</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>09/2026</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>NV0904</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Ms. Vân</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>09/2026</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>NV2412</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ms. Trâm</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>09/2026</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>NV2301</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Ms. Uyên Vi</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>09/2026</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>NV0801</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Mr. Khôi</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>09/2026</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Ghi chú: số liệu trang này copy từ trang báo cáo web (?page=baocao).</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>